<commit_message>
Portal discovery, regional filtering, error handling and E2E tracking
</commit_message>
<xml_diff>
--- a/outputs/e2e-testing/E2E-TEST-TRACKER.xlsx
+++ b/outputs/e2e-testing/E2E-TEST-TRACKER.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb9b0ca889a1241e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Register" sheetId="2" r:id="Rba8a2dbc45cd4726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="3" r:id="Rf5f02e3f80744d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R93ed0f2f48a544cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Checks" sheetId="5" r:id="Rd3e1ef9dab9b40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="6" r:id="Rb51b9808caa24761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists &amp; Config" sheetId="7" r:id="Rb850e3db37044824"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5dafdc1e154f4712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Register" sheetId="2" r:id="Rbe24463c8e894590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="3" r:id="R9d4f9a462fa44b9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R2c1af0f23fb94d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Checks" sheetId="5" r:id="Rc1afa44e317c4950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="6" r:id="Rd1376a9d96ab4d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists &amp; Config" sheetId="7" r:id="R3cd5fbac2517492a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -178,7 +178,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -301,6 +301,9 @@
     <x:xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -312,7 +315,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -323,7 +326,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +337,7 @@
         <x:color rgb="FF216E4E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFFF1"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +348,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +359,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -366,7 +369,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7D6"/>
         </x:patternFill>
       </x:fill>
@@ -377,7 +380,7 @@
         <x:color rgb="FF0C66E4"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F2FF"/>
         </x:patternFill>
       </x:fill>
@@ -388,7 +391,7 @@
         <x:color rgb="FF216E4E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFFF1"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +402,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +413,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -420,7 +423,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7D6"/>
         </x:patternFill>
       </x:fill>
@@ -431,7 +434,7 @@
         <x:color rgb="FF0C66E4"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F2FF"/>
         </x:patternFill>
       </x:fill>
@@ -442,7 +445,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFBDAD"/>
         </x:patternFill>
       </x:fill>
@@ -453,7 +456,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -464,7 +467,7 @@
         <x:color rgb="FF216E4E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFFF1"/>
         </x:patternFill>
       </x:fill>
@@ -475,7 +478,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -486,7 +489,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -496,7 +499,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7D6"/>
         </x:patternFill>
       </x:fill>
@@ -507,7 +510,7 @@
         <x:color rgb="FF0C66E4"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F2FF"/>
         </x:patternFill>
       </x:fill>
@@ -518,7 +521,7 @@
         <x:color rgb="FF216E4E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFFF1"/>
         </x:patternFill>
       </x:fill>
@@ -529,7 +532,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -540,7 +543,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -550,7 +553,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7D6"/>
         </x:patternFill>
       </x:fill>
@@ -561,7 +564,7 @@
         <x:color rgb="FF0C66E4"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F2FF"/>
         </x:patternFill>
       </x:fill>
@@ -572,7 +575,7 @@
         <x:color rgb="FF216E4E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFFF1"/>
         </x:patternFill>
       </x:fill>
@@ -583,7 +586,7 @@
         <x:color rgb="FFAE2A19"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFECEB"/>
         </x:patternFill>
       </x:fill>
@@ -594,7 +597,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF3E0"/>
         </x:patternFill>
       </x:fill>
@@ -604,7 +607,7 @@
         <x:color rgb="FF974F0C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7D6"/>
         </x:patternFill>
       </x:fill>
@@ -615,7 +618,7 @@
         <x:color rgb="FF0C66E4"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9F2FF"/>
         </x:patternFill>
       </x:fill>
@@ -825,7 +828,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb5f8a01c48404e47"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4f89dd0203340d1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -855,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re66106a7dd9a43c0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R70729041dc8446e8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -926,8 +929,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:AD6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AD6"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:AD18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AD18"/>
   <x:tableColumns count="30">
     <x:tableColumn id="1" name="Defect ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1307,7 +1310,7 @@
       </x:c>
       <x:c r="E5" s="48" t="n">
         <x:f>COUNTIF('Defects'!$K$6:$K$505,"New")+COUNTIF('Defects'!$K$6:$K$505,"Triaged")+COUNTIF('Defects'!$K$6:$K$505,"In Progress")+COUNTIF('Defects'!$K$6:$K$505,"Ready for Retest")+COUNTIF('Defects'!$K$6:$K$505,"Reopened")+COUNTIF('Defects'!$K$6:$K$505,"Blocked")</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="34"/>
       <x:c r="G5" s="34"/>
@@ -1324,7 +1327,7 @@
       </x:c>
       <x:c r="B6" s="48" t="n">
         <x:f>COUNTIFS('Test Executions'!$K$6:$K$505,"&lt;&gt;Not Run",'Test Executions'!$K$6:$K$505,"&lt;&gt;")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="34"/>
       <x:c r="D6" s="47" t="str">
@@ -1332,7 +1335,7 @@
       </x:c>
       <x:c r="E6" s="48" t="n">
         <x:f>COUNTIFS('Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$I$6:$I$505,"P0",'Defects'!$K$6:$K$505,"&lt;&gt;Closed")+COUNTIFS('Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$I$6:$I$505,"P1",'Defects'!$K$6:$K$505,"&lt;&gt;Closed")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F6" s="34"/>
       <x:c r="G6" s="34"/>
@@ -1357,7 +1360,7 @@
       </x:c>
       <x:c r="E7" s="48" t="n">
         <x:f>COUNTIF('Defects'!$K$6:$K$505,"Ready for Retest")</x:f>
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F7" s="34"/>
       <x:c r="G7" s="34"/>
@@ -1516,7 +1519,7 @@
       </x:c>
       <x:c r="B15" s="53" t="n">
         <x:f>COUNTIF('Test Executions'!$K$6:$K$505,"Not Run")</x:f>
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C15" s="34"/>
       <x:c r="D15" s="53" t="str">
@@ -1541,7 +1544,7 @@
       </x:c>
       <x:c r="B16" s="53" t="n">
         <x:f>COUNTIF('Test Executions'!$K$6:$K$505,"In Progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="34"/>
       <x:c r="D16" s="53" t="str">
@@ -1549,7 +1552,7 @@
       </x:c>
       <x:c r="E16" s="53" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P1",'Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$K$6:$K$505,"&lt;&gt;Resolved")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F16" s="34"/>
       <x:c r="G16" s="34"/>
@@ -1574,7 +1577,7 @@
       </x:c>
       <x:c r="E17" s="53" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P2",'Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$K$6:$K$505,"&lt;&gt;Resolved")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F17" s="34"/>
       <x:c r="G17" s="34"/>
@@ -1643,7 +1646,7 @@
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea1ca73ac2aa4ed5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra172802743de41f8"/>
 </x:worksheet>
 </file>
 
@@ -7325,7 +7328,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68af697bd0944e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3e212d7cfd49a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8004,17 +8007,21 @@
       <x:c r="G14" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H14" s="39" t="str"/>
-      <x:c r="I14" s="43" t="str"/>
+      <x:c r="H14" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I14" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J14" s="43" t="str"/>
       <x:c r="K14" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L14" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M14" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N14" s="39" t="str">
         <x:v>Pending</x:v>
@@ -8028,14 +8035,20 @@
       <x:c r="Q14" s="41" t="str"/>
       <x:c r="R14" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C14)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S14" s="39" t="str"/>
-      <x:c r="T14" s="39" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S14" s="39" t="str">
+        <x:v>BUG-0002, BUG-0003, BUG-0004</x:v>
+      </x:c>
+      <x:c r="T14" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U14" s="39" t="str"/>
       <x:c r="V14" s="39" t="str"/>
       <x:c r="W14" s="39" t="str"/>
-      <x:c r="X14" s="39" t="str"/>
+      <x:c r="X14" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="39" t="str">
@@ -8059,17 +8072,21 @@
       <x:c r="G15" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H15" s="39" t="str"/>
-      <x:c r="I15" s="43" t="str"/>
+      <x:c r="H15" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I15" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J15" s="43" t="str"/>
       <x:c r="K15" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L15" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M15" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N15" s="39" t="str">
         <x:v>Pending</x:v>
@@ -8083,14 +8100,20 @@
       <x:c r="Q15" s="41" t="str"/>
       <x:c r="R15" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C15)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S15" s="39" t="str"/>
-      <x:c r="T15" s="39" t="str"/>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="S15" s="39" t="str">
+        <x:v>BUG-0005, BUG-0006</x:v>
+      </x:c>
+      <x:c r="T15" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U15" s="39" t="str"/>
       <x:c r="V15" s="39" t="str"/>
       <x:c r="W15" s="39" t="str"/>
-      <x:c r="X15" s="39" t="str"/>
+      <x:c r="X15" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="39" t="str">
@@ -8169,17 +8192,21 @@
       <x:c r="G17" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H17" s="39" t="str"/>
-      <x:c r="I17" s="43" t="str"/>
+      <x:c r="H17" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I17" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J17" s="43" t="str"/>
       <x:c r="K17" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L17" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M17" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N17" s="39" t="str">
         <x:v>Not Applicable</x:v>
@@ -8193,14 +8220,20 @@
       <x:c r="Q17" s="41" t="str"/>
       <x:c r="R17" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C17)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S17" s="39" t="str"/>
-      <x:c r="T17" s="39" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S17" s="39" t="str">
+        <x:v>BUG-0007</x:v>
+      </x:c>
+      <x:c r="T17" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U17" s="39" t="str"/>
       <x:c r="V17" s="39" t="str"/>
       <x:c r="W17" s="39" t="str"/>
-      <x:c r="X17" s="39" t="str"/>
+      <x:c r="X17" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="39" t="str">
@@ -8279,17 +8312,21 @@
       <x:c r="G19" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H19" s="39" t="str"/>
-      <x:c r="I19" s="43" t="str"/>
+      <x:c r="H19" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I19" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J19" s="43" t="str"/>
       <x:c r="K19" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L19" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M19" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N19" s="39" t="str">
         <x:v>Pending</x:v>
@@ -8303,14 +8340,20 @@
       <x:c r="Q19" s="41" t="str"/>
       <x:c r="R19" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C19)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S19" s="39" t="str"/>
-      <x:c r="T19" s="39" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S19" s="39" t="str">
+        <x:v>BUG-0001</x:v>
+      </x:c>
+      <x:c r="T19" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U19" s="39" t="str"/>
       <x:c r="V19" s="39" t="str"/>
       <x:c r="W19" s="39" t="str"/>
-      <x:c r="X19" s="39" t="str"/>
+      <x:c r="X19" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="39" t="str">
@@ -9104,17 +9147,21 @@
       <x:c r="G34" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H34" s="39" t="str"/>
-      <x:c r="I34" s="43" t="str"/>
+      <x:c r="H34" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I34" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J34" s="43" t="str"/>
       <x:c r="K34" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L34" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M34" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N34" s="39" t="str">
         <x:v>Pending</x:v>
@@ -9128,14 +9175,20 @@
       <x:c r="Q34" s="41" t="str"/>
       <x:c r="R34" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C34)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S34" s="39" t="str"/>
-      <x:c r="T34" s="39" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S34" s="39" t="str">
+        <x:v>BUG-0013</x:v>
+      </x:c>
+      <x:c r="T34" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U34" s="39" t="str"/>
       <x:c r="V34" s="39" t="str"/>
       <x:c r="W34" s="39" t="str"/>
-      <x:c r="X34" s="39" t="str"/>
+      <x:c r="X34" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="39" t="str">
@@ -9214,17 +9267,21 @@
       <x:c r="G36" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H36" s="39" t="str"/>
-      <x:c r="I36" s="43" t="str"/>
+      <x:c r="H36" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I36" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J36" s="43" t="str"/>
       <x:c r="K36" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L36" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M36" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N36" s="39" t="str">
         <x:v>Pending</x:v>
@@ -9238,14 +9295,20 @@
       <x:c r="Q36" s="41" t="str"/>
       <x:c r="R36" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C36)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S36" s="39" t="str"/>
-      <x:c r="T36" s="39" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S36" s="39" t="str">
+        <x:v>BUG-0012</x:v>
+      </x:c>
+      <x:c r="T36" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U36" s="39" t="str"/>
       <x:c r="V36" s="39" t="str"/>
       <x:c r="W36" s="39" t="str"/>
-      <x:c r="X36" s="39" t="str"/>
+      <x:c r="X36" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="39" t="str">
@@ -10369,17 +10432,21 @@
       <x:c r="G57" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H57" s="39" t="str"/>
-      <x:c r="I57" s="43" t="str"/>
+      <x:c r="H57" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I57" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J57" s="43" t="str"/>
       <x:c r="K57" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L57" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M57" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N57" s="39" t="str">
         <x:v>Pending</x:v>
@@ -10393,14 +10460,20 @@
       <x:c r="Q57" s="41" t="str"/>
       <x:c r="R57" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C57)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S57" s="39" t="str"/>
-      <x:c r="T57" s="39" t="str"/>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="S57" s="39" t="str">
+        <x:v>BUG-0008</x:v>
+      </x:c>
+      <x:c r="T57" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U57" s="39" t="str"/>
       <x:c r="V57" s="39" t="str"/>
       <x:c r="W57" s="39" t="str"/>
-      <x:c r="X57" s="39" t="str"/>
+      <x:c r="X57" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="39" t="str">
@@ -10754,17 +10827,21 @@
       <x:c r="G64" s="39" t="str">
         <x:v>Desktop 1440px</x:v>
       </x:c>
-      <x:c r="H64" s="39" t="str"/>
-      <x:c r="I64" s="43" t="str"/>
+      <x:c r="H64" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="I64" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
       <x:c r="J64" s="43" t="str"/>
       <x:c r="K64" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="L64" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="M64" s="39" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Partially Passed</x:v>
       </x:c>
       <x:c r="N64" s="39" t="str">
         <x:v>Pending</x:v>
@@ -10778,14 +10855,20 @@
       <x:c r="Q64" s="41" t="str"/>
       <x:c r="R64" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C64)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S64" s="39" t="str"/>
-      <x:c r="T64" s="39" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="S64" s="39" t="str">
+        <x:v>BUG-0009, BUG-0010, BUG-0011</x:v>
+      </x:c>
+      <x:c r="T64" s="39" t="str">
+        <x:v>Manual local E2E; see linked Defects rows</x:v>
+      </x:c>
       <x:c r="U64" s="39" t="str"/>
       <x:c r="V64" s="39" t="str"/>
       <x:c r="W64" s="39" t="str"/>
-      <x:c r="X64" s="39" t="str"/>
+      <x:c r="X64" s="39" t="str">
+        <x:v>Defects fixed; complete the remaining flow and inline DB checks before marking Passed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="39" t="str">
@@ -12676,7 +12759,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R102ecb00424741dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0412d6ce7e6d4b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12941,421 +13024,1149 @@
         <x:v>Resolution</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="39" t="str"/>
-      <x:c r="B6" s="39" t="str"/>
-      <x:c r="C6" s="39" t="str"/>
-      <x:c r="D6" s="39" t="str"/>
-      <x:c r="E6" s="39" t="str"/>
-      <x:c r="F6" s="39" t="str"/>
-      <x:c r="G6" s="39" t="str"/>
-      <x:c r="H6" s="39" t="str"/>
-      <x:c r="I6" s="39" t="str"/>
-      <x:c r="J6" s="39" t="str"/>
-      <x:c r="K6" s="39" t="str"/>
-      <x:c r="L6" s="39" t="str"/>
-      <x:c r="M6" s="39" t="str"/>
-      <x:c r="N6" s="39" t="str"/>
-      <x:c r="O6" s="39" t="str"/>
-      <x:c r="P6" s="43" t="str"/>
-      <x:c r="Q6" s="41" t="str"/>
-      <x:c r="R6" s="41" t="str"/>
-      <x:c r="S6" s="41" t="str"/>
-      <x:c r="T6" s="41" t="str"/>
-      <x:c r="U6" s="39" t="str"/>
-      <x:c r="V6" s="39" t="str"/>
-      <x:c r="W6" s="39" t="str"/>
-      <x:c r="X6" s="39" t="str"/>
-      <x:c r="Y6" s="39" t="str"/>
-      <x:c r="Z6" s="39" t="str"/>
-      <x:c r="AA6" s="39" t="str"/>
-      <x:c r="AB6" s="39" t="str"/>
-      <x:c r="AC6" s="43" t="str"/>
-      <x:c r="AD6" s="39" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="39"/>
-      <x:c r="B7" s="39"/>
-      <x:c r="C7" s="39"/>
-      <x:c r="D7" s="39"/>
-      <x:c r="E7" s="39"/>
-      <x:c r="F7" s="39"/>
-      <x:c r="G7" s="39"/>
-      <x:c r="H7" s="39"/>
-      <x:c r="I7" s="39"/>
-      <x:c r="J7" s="39"/>
-      <x:c r="K7" s="39"/>
-      <x:c r="L7" s="39"/>
-      <x:c r="M7" s="39"/>
-      <x:c r="N7" s="39"/>
-      <x:c r="O7" s="39"/>
-      <x:c r="P7" s="43"/>
-      <x:c r="Q7" s="41"/>
-      <x:c r="R7" s="41"/>
-      <x:c r="S7" s="41"/>
-      <x:c r="T7" s="41"/>
-      <x:c r="U7" s="39"/>
-      <x:c r="V7" s="39"/>
-      <x:c r="W7" s="39"/>
-      <x:c r="X7" s="39"/>
-      <x:c r="Y7" s="39"/>
-      <x:c r="Z7" s="39"/>
-      <x:c r="AA7" s="39"/>
-      <x:c r="AB7" s="39"/>
-      <x:c r="AC7" s="43"/>
-      <x:c r="AD7" s="39"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="39"/>
-      <x:c r="B8" s="39"/>
-      <x:c r="C8" s="39"/>
-      <x:c r="D8" s="39"/>
-      <x:c r="E8" s="39"/>
-      <x:c r="F8" s="39"/>
-      <x:c r="G8" s="39"/>
-      <x:c r="H8" s="39"/>
-      <x:c r="I8" s="39"/>
-      <x:c r="J8" s="39"/>
-      <x:c r="K8" s="39"/>
-      <x:c r="L8" s="39"/>
-      <x:c r="M8" s="39"/>
-      <x:c r="N8" s="39"/>
-      <x:c r="O8" s="39"/>
-      <x:c r="P8" s="43"/>
-      <x:c r="Q8" s="41"/>
-      <x:c r="R8" s="41"/>
-      <x:c r="S8" s="41"/>
-      <x:c r="T8" s="41"/>
-      <x:c r="U8" s="39"/>
-      <x:c r="V8" s="39"/>
-      <x:c r="W8" s="39"/>
-      <x:c r="X8" s="39"/>
-      <x:c r="Y8" s="39"/>
-      <x:c r="Z8" s="39"/>
-      <x:c r="AA8" s="39"/>
-      <x:c r="AB8" s="39"/>
-      <x:c r="AC8" s="43"/>
-      <x:c r="AD8" s="39"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="39"/>
-      <x:c r="B9" s="39"/>
-      <x:c r="C9" s="39"/>
-      <x:c r="D9" s="39"/>
-      <x:c r="E9" s="39"/>
-      <x:c r="F9" s="39"/>
-      <x:c r="G9" s="39"/>
-      <x:c r="H9" s="39"/>
-      <x:c r="I9" s="39"/>
-      <x:c r="J9" s="39"/>
-      <x:c r="K9" s="39"/>
-      <x:c r="L9" s="39"/>
-      <x:c r="M9" s="39"/>
-      <x:c r="N9" s="39"/>
-      <x:c r="O9" s="39"/>
-      <x:c r="P9" s="43"/>
-      <x:c r="Q9" s="41"/>
-      <x:c r="R9" s="41"/>
-      <x:c r="S9" s="41"/>
-      <x:c r="T9" s="41"/>
-      <x:c r="U9" s="39"/>
-      <x:c r="V9" s="39"/>
-      <x:c r="W9" s="39"/>
-      <x:c r="X9" s="39"/>
-      <x:c r="Y9" s="39"/>
-      <x:c r="Z9" s="39"/>
-      <x:c r="AA9" s="39"/>
-      <x:c r="AB9" s="39"/>
-      <x:c r="AC9" s="43"/>
-      <x:c r="AD9" s="39"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="39"/>
-      <x:c r="B10" s="39"/>
-      <x:c r="C10" s="39"/>
-      <x:c r="D10" s="39"/>
-      <x:c r="E10" s="39"/>
-      <x:c r="F10" s="39"/>
-      <x:c r="G10" s="39"/>
-      <x:c r="H10" s="39"/>
-      <x:c r="I10" s="39"/>
-      <x:c r="J10" s="39"/>
-      <x:c r="K10" s="39"/>
-      <x:c r="L10" s="39"/>
-      <x:c r="M10" s="39"/>
-      <x:c r="N10" s="39"/>
-      <x:c r="O10" s="39"/>
-      <x:c r="P10" s="43"/>
-      <x:c r="Q10" s="41"/>
-      <x:c r="R10" s="41"/>
-      <x:c r="S10" s="41"/>
-      <x:c r="T10" s="41"/>
-      <x:c r="U10" s="39"/>
-      <x:c r="V10" s="39"/>
-      <x:c r="W10" s="39"/>
-      <x:c r="X10" s="39"/>
-      <x:c r="Y10" s="39"/>
-      <x:c r="Z10" s="39"/>
-      <x:c r="AA10" s="39"/>
-      <x:c r="AB10" s="39"/>
-      <x:c r="AC10" s="43"/>
-      <x:c r="AD10" s="39"/>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="39"/>
-      <x:c r="B11" s="39"/>
-      <x:c r="C11" s="39"/>
-      <x:c r="D11" s="39"/>
-      <x:c r="E11" s="39"/>
-      <x:c r="F11" s="39"/>
-      <x:c r="G11" s="39"/>
-      <x:c r="H11" s="39"/>
-      <x:c r="I11" s="39"/>
-      <x:c r="J11" s="39"/>
-      <x:c r="K11" s="39"/>
-      <x:c r="L11" s="39"/>
-      <x:c r="M11" s="39"/>
-      <x:c r="N11" s="39"/>
-      <x:c r="O11" s="39"/>
-      <x:c r="P11" s="43"/>
-      <x:c r="Q11" s="41"/>
-      <x:c r="R11" s="41"/>
-      <x:c r="S11" s="41"/>
-      <x:c r="T11" s="41"/>
-      <x:c r="U11" s="39"/>
-      <x:c r="V11" s="39"/>
-      <x:c r="W11" s="39"/>
-      <x:c r="X11" s="39"/>
-      <x:c r="Y11" s="39"/>
-      <x:c r="Z11" s="39"/>
-      <x:c r="AA11" s="39"/>
-      <x:c r="AB11" s="39"/>
-      <x:c r="AC11" s="43"/>
-      <x:c r="AD11" s="39"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="39"/>
-      <x:c r="B12" s="39"/>
-      <x:c r="C12" s="39"/>
-      <x:c r="D12" s="39"/>
-      <x:c r="E12" s="39"/>
-      <x:c r="F12" s="39"/>
-      <x:c r="G12" s="39"/>
-      <x:c r="H12" s="39"/>
-      <x:c r="I12" s="39"/>
-      <x:c r="J12" s="39"/>
-      <x:c r="K12" s="39"/>
-      <x:c r="L12" s="39"/>
-      <x:c r="M12" s="39"/>
-      <x:c r="N12" s="39"/>
-      <x:c r="O12" s="39"/>
-      <x:c r="P12" s="43"/>
-      <x:c r="Q12" s="41"/>
-      <x:c r="R12" s="41"/>
-      <x:c r="S12" s="41"/>
-      <x:c r="T12" s="41"/>
-      <x:c r="U12" s="39"/>
-      <x:c r="V12" s="39"/>
-      <x:c r="W12" s="39"/>
-      <x:c r="X12" s="39"/>
-      <x:c r="Y12" s="39"/>
-      <x:c r="Z12" s="39"/>
-      <x:c r="AA12" s="39"/>
-      <x:c r="AB12" s="39"/>
-      <x:c r="AC12" s="43"/>
-      <x:c r="AD12" s="39"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="39"/>
-      <x:c r="B13" s="39"/>
-      <x:c r="C13" s="39"/>
-      <x:c r="D13" s="39"/>
-      <x:c r="E13" s="39"/>
-      <x:c r="F13" s="39"/>
-      <x:c r="G13" s="39"/>
-      <x:c r="H13" s="39"/>
-      <x:c r="I13" s="39"/>
-      <x:c r="J13" s="39"/>
-      <x:c r="K13" s="39"/>
-      <x:c r="L13" s="39"/>
-      <x:c r="M13" s="39"/>
-      <x:c r="N13" s="39"/>
-      <x:c r="O13" s="39"/>
-      <x:c r="P13" s="43"/>
-      <x:c r="Q13" s="41"/>
-      <x:c r="R13" s="41"/>
-      <x:c r="S13" s="41"/>
-      <x:c r="T13" s="41"/>
-      <x:c r="U13" s="39"/>
-      <x:c r="V13" s="39"/>
-      <x:c r="W13" s="39"/>
-      <x:c r="X13" s="39"/>
-      <x:c r="Y13" s="39"/>
-      <x:c r="Z13" s="39"/>
-      <x:c r="AA13" s="39"/>
-      <x:c r="AB13" s="39"/>
-      <x:c r="AC13" s="43"/>
-      <x:c r="AD13" s="39"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="39"/>
-      <x:c r="B14" s="39"/>
-      <x:c r="C14" s="39"/>
-      <x:c r="D14" s="39"/>
-      <x:c r="E14" s="39"/>
-      <x:c r="F14" s="39"/>
-      <x:c r="G14" s="39"/>
-      <x:c r="H14" s="39"/>
-      <x:c r="I14" s="39"/>
-      <x:c r="J14" s="39"/>
-      <x:c r="K14" s="39"/>
-      <x:c r="L14" s="39"/>
-      <x:c r="M14" s="39"/>
-      <x:c r="N14" s="39"/>
-      <x:c r="O14" s="39"/>
-      <x:c r="P14" s="43"/>
-      <x:c r="Q14" s="41"/>
-      <x:c r="R14" s="41"/>
-      <x:c r="S14" s="41"/>
-      <x:c r="T14" s="41"/>
-      <x:c r="U14" s="39"/>
-      <x:c r="V14" s="39"/>
-      <x:c r="W14" s="39"/>
-      <x:c r="X14" s="39"/>
-      <x:c r="Y14" s="39"/>
-      <x:c r="Z14" s="39"/>
-      <x:c r="AA14" s="39"/>
-      <x:c r="AB14" s="39"/>
-      <x:c r="AC14" s="43"/>
-      <x:c r="AD14" s="39"/>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="39"/>
-      <x:c r="B15" s="39"/>
-      <x:c r="C15" s="39"/>
-      <x:c r="D15" s="39"/>
-      <x:c r="E15" s="39"/>
-      <x:c r="F15" s="39"/>
-      <x:c r="G15" s="39"/>
-      <x:c r="H15" s="39"/>
-      <x:c r="I15" s="39"/>
-      <x:c r="J15" s="39"/>
-      <x:c r="K15" s="39"/>
-      <x:c r="L15" s="39"/>
-      <x:c r="M15" s="39"/>
-      <x:c r="N15" s="39"/>
-      <x:c r="O15" s="39"/>
-      <x:c r="P15" s="43"/>
-      <x:c r="Q15" s="41"/>
-      <x:c r="R15" s="41"/>
-      <x:c r="S15" s="41"/>
-      <x:c r="T15" s="41"/>
-      <x:c r="U15" s="39"/>
-      <x:c r="V15" s="39"/>
-      <x:c r="W15" s="39"/>
-      <x:c r="X15" s="39"/>
-      <x:c r="Y15" s="39"/>
-      <x:c r="Z15" s="39"/>
-      <x:c r="AA15" s="39"/>
-      <x:c r="AB15" s="39"/>
-      <x:c r="AC15" s="43"/>
-      <x:c r="AD15" s="39"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="39"/>
-      <x:c r="B16" s="39"/>
-      <x:c r="C16" s="39"/>
-      <x:c r="D16" s="39"/>
-      <x:c r="E16" s="39"/>
-      <x:c r="F16" s="39"/>
-      <x:c r="G16" s="39"/>
-      <x:c r="H16" s="39"/>
-      <x:c r="I16" s="39"/>
-      <x:c r="J16" s="39"/>
-      <x:c r="K16" s="39"/>
-      <x:c r="L16" s="39"/>
-      <x:c r="M16" s="39"/>
-      <x:c r="N16" s="39"/>
-      <x:c r="O16" s="39"/>
-      <x:c r="P16" s="43"/>
-      <x:c r="Q16" s="41"/>
-      <x:c r="R16" s="41"/>
-      <x:c r="S16" s="41"/>
-      <x:c r="T16" s="41"/>
-      <x:c r="U16" s="39"/>
-      <x:c r="V16" s="39"/>
-      <x:c r="W16" s="39"/>
-      <x:c r="X16" s="39"/>
-      <x:c r="Y16" s="39"/>
-      <x:c r="Z16" s="39"/>
-      <x:c r="AA16" s="39"/>
-      <x:c r="AB16" s="39"/>
-      <x:c r="AC16" s="43"/>
-      <x:c r="AD16" s="39"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="39"/>
-      <x:c r="B17" s="39"/>
-      <x:c r="C17" s="39"/>
-      <x:c r="D17" s="39"/>
-      <x:c r="E17" s="39"/>
-      <x:c r="F17" s="39"/>
-      <x:c r="G17" s="39"/>
-      <x:c r="H17" s="39"/>
-      <x:c r="I17" s="39"/>
-      <x:c r="J17" s="39"/>
-      <x:c r="K17" s="39"/>
-      <x:c r="L17" s="39"/>
-      <x:c r="M17" s="39"/>
-      <x:c r="N17" s="39"/>
-      <x:c r="O17" s="39"/>
-      <x:c r="P17" s="43"/>
-      <x:c r="Q17" s="41"/>
-      <x:c r="R17" s="41"/>
-      <x:c r="S17" s="41"/>
-      <x:c r="T17" s="41"/>
-      <x:c r="U17" s="39"/>
-      <x:c r="V17" s="39"/>
-      <x:c r="W17" s="39"/>
-      <x:c r="X17" s="39"/>
-      <x:c r="Y17" s="39"/>
-      <x:c r="Z17" s="39"/>
-      <x:c r="AA17" s="39"/>
-      <x:c r="AB17" s="39"/>
-      <x:c r="AC17" s="43"/>
-      <x:c r="AD17" s="39"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="39"/>
-      <x:c r="B18" s="39"/>
-      <x:c r="C18" s="39"/>
-      <x:c r="D18" s="39"/>
-      <x:c r="E18" s="39"/>
-      <x:c r="F18" s="39"/>
-      <x:c r="G18" s="39"/>
-      <x:c r="H18" s="39"/>
-      <x:c r="I18" s="39"/>
-      <x:c r="J18" s="39"/>
-      <x:c r="K18" s="39"/>
-      <x:c r="L18" s="39"/>
-      <x:c r="M18" s="39"/>
-      <x:c r="N18" s="39"/>
-      <x:c r="O18" s="39"/>
-      <x:c r="P18" s="43"/>
-      <x:c r="Q18" s="41"/>
-      <x:c r="R18" s="41"/>
-      <x:c r="S18" s="41"/>
-      <x:c r="T18" s="41"/>
-      <x:c r="U18" s="39"/>
-      <x:c r="V18" s="39"/>
-      <x:c r="W18" s="39"/>
-      <x:c r="X18" s="39"/>
-      <x:c r="Y18" s="39"/>
-      <x:c r="Z18" s="39"/>
-      <x:c r="AA18" s="39"/>
-      <x:c r="AB18" s="39"/>
-      <x:c r="AC18" s="43"/>
-      <x:c r="AD18" s="39"/>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="41" t="str">
+        <x:v>BUG-0001</x:v>
+      </x:c>
+      <x:c r="B6" s="41" t="str">
+        <x:v>Landing pages entered repeated render and query cycles</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>EVT-001</x:v>
+      </x:c>
+      <x:c r="D6" s="41" t="str">
+        <x:v>EXEC-0014</x:v>
+      </x:c>
+      <x:c r="E6" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F6" s="41" t="str">
+        <x:v>Events / Jobs / Marketplace</x:v>
+      </x:c>
+      <x:c r="G6" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H6" s="41" t="str">
+        <x:v>Apollo page queries</x:v>
+      </x:c>
+      <x:c r="I6" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J6" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K6" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L6" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M6" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N6" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O6" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P6" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q6" s="41" t="str">
+        <x:v>Opening a browse landing page caused Maximum update depth errors and repeated Apollo requests.</x:v>
+      </x:c>
+      <x:c r="R6" s="41" t="str">
+        <x:v>Open /events, /jobs, or /marketplace and observe repeated renders/network calls.</x:v>
+      </x:c>
+      <x:c r="S6" s="41" t="str">
+        <x:v>Each page renders once and refetches only when stable filter inputs change.</x:v>
+      </x:c>
+      <x:c r="T6" s="41" t="str">
+        <x:v>Unstable date variables and newly allocated empty preference arrays retriggered query/render work.</x:v>
+      </x:c>
+      <x:c r="U6" s="41" t="str">
+        <x:v>Browser console; apps/christian-listing/src/pages/EventsPage.tsx</x:v>
+      </x:c>
+      <x:c r="V6" s="41"/>
+      <x:c r="W6" s="41"/>
+      <x:c r="X6" s="41" t="str">
+        <x:v>Render-time query variables and selector fallbacks changed identity on every render.</x:v>
+      </x:c>
+      <x:c r="Y6" s="41" t="str">
+        <x:v>54ad9af</x:v>
+      </x:c>
+      <x:c r="Z6" s="41" t="str">
+        <x:v>54ad9af</x:v>
+      </x:c>
+      <x:c r="AA6" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB6" s="41" t="str">
+        <x:v>EXEC-0014</x:v>
+      </x:c>
+      <x:c r="AC6" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD6" s="41" t="str">
+        <x:v>Memoised date variables and shared stable empty arrays across the three landing pages.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>BUG-0002</x:v>
+      </x:c>
+      <x:c r="B7" s="41" t="str">
+        <x:v>Homepage discovery sections used hardcoded content</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>DISC-001</x:v>
+      </x:c>
+      <x:c r="D7" s="41" t="str">
+        <x:v>EXEC-0009</x:v>
+      </x:c>
+      <x:c r="E7" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F7" s="41" t="str">
+        <x:v>Discovery</x:v>
+      </x:c>
+      <x:c r="G7" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H7" s="41" t="str">
+        <x:v>Spotlight and Events at a Glance</x:v>
+      </x:c>
+      <x:c r="I7" s="41" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J7" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K7" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L7" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M7" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N7" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O7" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P7" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q7" s="41" t="str">
+        <x:v>Spotlight and Events at a Glance displayed static fixture cards instead of published platform content.</x:v>
+      </x:c>
+      <x:c r="R7" s="41" t="str">
+        <x:v>Open / and compare section cards with current published event, job, and listing records.</x:v>
+      </x:c>
+      <x:c r="S7" s="41" t="str">
+        <x:v>Sections select current published content, prioritising the selected region.</x:v>
+      </x:c>
+      <x:c r="T7" s="41" t="str">
+        <x:v>Static JSX and asset data were used by both sections.</x:v>
+      </x:c>
+      <x:c r="U7" s="41" t="str">
+        <x:v>apps/christian-listing/src/lib/homepage.ts; homepage-selection.spec.ts</x:v>
+      </x:c>
+      <x:c r="V7" s="41"/>
+      <x:c r="W7" s="41"/>
+      <x:c r="X7" s="41" t="str">
+        <x:v>Homepage sections had no shared live discovery selection layer.</x:v>
+      </x:c>
+      <x:c r="Y7" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z7" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA7" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB7" s="41"/>
+      <x:c r="AC7" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD7" s="41" t="str">
+        <x:v>Added a live homepage query and deterministic selection logic for spotlight and event-glance content.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="41" t="str">
+        <x:v>BUG-0003</x:v>
+      </x:c>
+      <x:c r="B8" s="41" t="str">
+        <x:v>Homepage failed to compile after Spotlight implementation</x:v>
+      </x:c>
+      <x:c r="C8" s="41" t="str">
+        <x:v>DISC-001</x:v>
+      </x:c>
+      <x:c r="D8" s="41" t="str">
+        <x:v>EXEC-0009</x:v>
+      </x:c>
+      <x:c r="E8" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F8" s="41" t="str">
+        <x:v>Discovery</x:v>
+      </x:c>
+      <x:c r="G8" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H8" s="41" t="str">
+        <x:v>Homepage Spotlight import</x:v>
+      </x:c>
+      <x:c r="I8" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J8" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K8" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L8" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M8" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N8" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O8" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P8" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q8" s="41" t="str">
+        <x:v>Webpack reported TS2307 for ../components/sections/SpotlightSection.</x:v>
+      </x:c>
+      <x:c r="R8" s="41" t="str">
+        <x:v>Start the web app after the homepage discovery change.</x:v>
+      </x:c>
+      <x:c r="S8" s="41" t="str">
+        <x:v>The homepage compiles and the Spotlight section renders.</x:v>
+      </x:c>
+      <x:c r="T8" s="41" t="str">
+        <x:v>Build stopped because the imported module path did not exist.</x:v>
+      </x:c>
+      <x:c r="U8" s="41" t="str">
+        <x:v>Compiler error TS2307; apps/christian-listing/src/pages/HomePage.tsx</x:v>
+      </x:c>
+      <x:c r="V8" s="41"/>
+      <x:c r="W8" s="41"/>
+      <x:c r="X8" s="41" t="str">
+        <x:v>The new component filename and HomePage import were inconsistent.</x:v>
+      </x:c>
+      <x:c r="Y8" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z8" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA8" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB8" s="41" t="str">
+        <x:v>EXEC-0009</x:v>
+      </x:c>
+      <x:c r="AC8" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD8" s="41" t="str">
+        <x:v>Added HomepageSpotlightSection and updated HomePage to import the actual module.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="41" t="str">
+        <x:v>BUG-0004</x:v>
+      </x:c>
+      <x:c r="B9" s="41" t="str">
+        <x:v>Regional discovery became blank when the selected location had no matches</x:v>
+      </x:c>
+      <x:c r="C9" s="41" t="str">
+        <x:v>DISC-001</x:v>
+      </x:c>
+      <x:c r="D9" s="41" t="str">
+        <x:v>EXEC-0009</x:v>
+      </x:c>
+      <x:c r="E9" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F9" s="41" t="str">
+        <x:v>Discovery</x:v>
+      </x:c>
+      <x:c r="G9" s="41" t="str">
+        <x:v>Backend Logic</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>Regional/global selection</x:v>
+      </x:c>
+      <x:c r="I9" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K9" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L9" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M9" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N9" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O9" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P9" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q9" s="41" t="str">
+        <x:v>With GB-LDN selected, discovery sections could show no content even when active content existed elsewhere.</x:v>
+      </x:c>
+      <x:c r="R9" s="41" t="str">
+        <x:v>Select GB-LDN, open /, and inspect Spotlight and other location-aware discovery sections.</x:v>
+      </x:c>
+      <x:c r="S9" s="41" t="str">
+        <x:v>Regional content appears first; remaining slots fall back to global active content.</x:v>
+      </x:c>
+      <x:c r="T9" s="41" t="str">
+        <x:v>The page displayed an empty regional result without a global fallback.</x:v>
+      </x:c>
+      <x:c r="U9" s="41" t="str">
+        <x:v>apps/christian-listing/src/lib/discovery.ts; region-helpers.spec.ts</x:v>
+      </x:c>
+      <x:c r="V9" s="41"/>
+      <x:c r="W9" s="41" t="str">
+        <x:v>Region GB-LDN</x:v>
+      </x:c>
+      <x:c r="X9" s="41" t="str">
+        <x:v>Queries and selectors treated regional filtering as an all-or-nothing content boundary.</x:v>
+      </x:c>
+      <x:c r="Y9" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z9" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA9" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB9" s="41"/>
+      <x:c r="AC9" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD9" s="41" t="str">
+        <x:v>Merged unique regional and global result sets, retaining regional priority and explicit-search behaviour.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="41" t="str">
+        <x:v>BUG-0005</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="str">
+        <x:v>Me query requested User.regionCode outside the federated contract</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:v>DISC-002</x:v>
+      </x:c>
+      <x:c r="D10" s="41" t="str">
+        <x:v>EXEC-0010</x:v>
+      </x:c>
+      <x:c r="E10" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F10" s="41" t="str">
+        <x:v>Identity / Discovery</x:v>
+      </x:c>
+      <x:c r="G10" s="41" t="str">
+        <x:v>API / GraphQL</x:v>
+      </x:c>
+      <x:c r="H10" s="41" t="str">
+        <x:v>User schema contract</x:v>
+      </x:c>
+      <x:c r="I10" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J10" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K10" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L10" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M10" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N10" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O10" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P10" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q10" s="41" t="str">
+        <x:v>The me operation failed GraphQL validation because User.regionCode was unavailable.</x:v>
+      </x:c>
+      <x:c r="R10" s="41" t="str">
+        <x:v>Load an authenticated route that issues the me query.</x:v>
+      </x:c>
+      <x:c r="S10" s="41" t="str">
+        <x:v>The operation validates and returns the user region fields consumed by the client.</x:v>
+      </x:c>
+      <x:c r="T10" s="41" t="str">
+        <x:v>GRAPHQL_VALIDATION_FAILED: Cannot query field regionCode on type User.</x:v>
+      </x:c>
+      <x:c r="U10" s="41" t="str">
+        <x:v>identity.graphql; generated GraphQL types</x:v>
+      </x:c>
+      <x:c r="V10" s="41"/>
+      <x:c r="W10" s="41"/>
+      <x:c r="X10" s="41" t="str">
+        <x:v>Client operation, identity schema, and composed federation contract were out of sync.</x:v>
+      </x:c>
+      <x:c r="Y10" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z10" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA10" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB10" s="41" t="str">
+        <x:v>EXEC-0010</x:v>
+      </x:c>
+      <x:c r="AC10" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD10" s="41" t="str">
+        <x:v>Aligned the identity schema/resolvers and regenerated consuming GraphQL types.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="41" t="str">
+        <x:v>BUG-0006</x:v>
+      </x:c>
+      <x:c r="B11" s="41" t="str">
+        <x:v>Discovery failed on null federated marketplace seller id</x:v>
+      </x:c>
+      <x:c r="C11" s="41" t="str">
+        <x:v>DISC-002</x:v>
+      </x:c>
+      <x:c r="D11" s="41" t="str">
+        <x:v>EXEC-0010</x:v>
+      </x:c>
+      <x:c r="E11" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F11" s="41" t="str">
+        <x:v>Discovery / Marketplace</x:v>
+      </x:c>
+      <x:c r="G11" s="41" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="H11" s="41" t="str">
+        <x:v>Federated User reference</x:v>
+      </x:c>
+      <x:c r="I11" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J11" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K11" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L11" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M11" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N11" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O11" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P11" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q11" s="41" t="str">
+        <x:v>Discovery returned data null when a seeded listing seller could not complete non-null User.id.</x:v>
+      </x:c>
+      <x:c r="R11" s="41" t="str">
+        <x:v>Run Discovery with globalListings and request seller { id isVerified }.</x:v>
+      </x:c>
+      <x:c r="S11" s="41" t="str">
+        <x:v>A stale optional relationship cannot null the entire discovery response.</x:v>
+      </x:c>
+      <x:c r="T11" s="41" t="str">
+        <x:v>Cannot return null for non-nullable field User.id at globalListings.edges[0].seller.id.</x:v>
+      </x:c>
+      <x:c r="U11" s="41" t="str">
+        <x:v>GraphQL Discovery response; apps/christian-listing/src/lib/discovery.ts</x:v>
+      </x:c>
+      <x:c r="V11" s="41"/>
+      <x:c r="W11" s="41" t="str">
+        <x:v>Seeded marketplace listing seller</x:v>
+      </x:c>
+      <x:c r="X11" s="41" t="str">
+        <x:v>Discovery selected seller fields it did not render and legacy seed references lacked a resolvable identity.</x:v>
+      </x:c>
+      <x:c r="Y11" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z11" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA11" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB11" s="41" t="str">
+        <x:v>EXEC-0010</x:v>
+      </x:c>
+      <x:c r="AC11" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD11" s="41" t="str">
+        <x:v>Removed the unused seller selection and hardened federated user-reference mapping.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="41" t="str">
+        <x:v>BUG-0007</x:v>
+      </x:c>
+      <x:c r="B12" s="41" t="str">
+        <x:v>Public detail pages were obscured by the fixed navbar</x:v>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:v>DISC-004</x:v>
+      </x:c>
+      <x:c r="D12" s="41" t="str">
+        <x:v>EXEC-0012</x:v>
+      </x:c>
+      <x:c r="E12" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F12" s="41" t="str">
+        <x:v>Navigation / Layout</x:v>
+      </x:c>
+      <x:c r="G12" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H12" s="41" t="str">
+        <x:v>Job detail and member profile</x:v>
+      </x:c>
+      <x:c r="I12" s="41" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J12" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K12" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L12" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M12" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N12" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O12" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P12" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q12" s="41" t="str">
+        <x:v>The job detail and profile content started at top: 0 beneath the fixed navbar.</x:v>
+      </x:c>
+      <x:c r="R12" s="41" t="str">
+        <x:v>Open /jobs/700000000000000000000032 and /profile at desktop width.</x:v>
+      </x:c>
+      <x:c r="S12" s="41" t="str">
+        <x:v>The first page content starts below the navbar.</x:v>
+      </x:c>
+      <x:c r="T12" s="41" t="str">
+        <x:v>Headings and breadcrumbs were partially covered by navigation.</x:v>
+      </x:c>
+      <x:c r="U12" s="41" t="str">
+        <x:v>Routes /jobs/700000000000000000000032 and /profile</x:v>
+      </x:c>
+      <x:c r="V12" s="41"/>
+      <x:c r="W12" s="41" t="str">
+        <x:v>Job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X12" s="41" t="str">
+        <x:v>Affected page shells did not reserve the fixed header height.</x:v>
+      </x:c>
+      <x:c r="Y12" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z12" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA12" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB12" s="41" t="str">
+        <x:v>EXEC-0012</x:v>
+      </x:c>
+      <x:c r="AC12" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD12" s="41" t="str">
+        <x:v>Added the standard top offset to the affected page containers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="41" t="str">
+        <x:v>BUG-0008</x:v>
+      </x:c>
+      <x:c r="B13" s="41" t="str">
+        <x:v>Saved Items Hub had no discoverable navigation entry</x:v>
+      </x:c>
+      <x:c r="C13" s="41" t="str">
+        <x:v>MEM-003</x:v>
+      </x:c>
+      <x:c r="D13" s="41" t="str">
+        <x:v>EXEC-0052</x:v>
+      </x:c>
+      <x:c r="E13" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F13" s="41" t="str">
+        <x:v>Member Dashboard</x:v>
+      </x:c>
+      <x:c r="G13" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H13" s="41" t="str">
+        <x:v>Desktop and mobile user menus</x:v>
+      </x:c>
+      <x:c r="I13" s="41" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J13" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K13" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L13" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M13" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N13" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O13" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P13" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q13" s="41" t="str">
+        <x:v>The /dashboard/saved route existed but users could not reach it from the primary authenticated navigation.</x:v>
+      </x:c>
+      <x:c r="R13" s="41" t="str">
+        <x:v>Sign in, open the avatar menu, and look for Saved Items.</x:v>
+      </x:c>
+      <x:c r="S13" s="41" t="str">
+        <x:v>Dashboard and Saved Items are available in desktop and mobile menus.</x:v>
+      </x:c>
+      <x:c r="T13" s="41" t="str">
+        <x:v>No menu action linked to the Saved Items Hub.</x:v>
+      </x:c>
+      <x:c r="U13" s="41" t="str">
+        <x:v>apps/christian-listing/src/components/layout/Navbar.tsx</x:v>
+      </x:c>
+      <x:c r="V13" s="41"/>
+      <x:c r="W13" s="41"/>
+      <x:c r="X13" s="41" t="str">
+        <x:v>The hub route was implemented without a navigation affordance.</x:v>
+      </x:c>
+      <x:c r="Y13" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z13" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA13" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB13" s="41"/>
+      <x:c r="AC13" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD13" s="41" t="str">
+        <x:v>Added Dashboard and Saved Items actions to both authenticated user menus.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="41" t="str">
+        <x:v>BUG-0009</x:v>
+      </x:c>
+      <x:c r="B14" s="41" t="str">
+        <x:v>Organisation profile failed on marketplaceListings federation field</x:v>
+      </x:c>
+      <x:c r="C14" s="41" t="str">
+        <x:v>ORG-005</x:v>
+      </x:c>
+      <x:c r="D14" s="41" t="str">
+        <x:v>EXEC-0059</x:v>
+      </x:c>
+      <x:c r="E14" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F14" s="41" t="str">
+        <x:v>Organisation Profile</x:v>
+      </x:c>
+      <x:c r="G14" s="41" t="str">
+        <x:v>API / GraphQL</x:v>
+      </x:c>
+      <x:c r="H14" s="41" t="str">
+        <x:v>Organisation.marketplaceListings</x:v>
+      </x:c>
+      <x:c r="I14" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J14" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K14" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L14" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M14" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N14" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O14" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P14" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q14" s="41" t="str">
+        <x:v>A seeded organisation existed, but its public profile failed with a non-null marketplaceListings completion error.</x:v>
+      </x:c>
+      <x:c r="R14" s="41" t="str">
+        <x:v>From the seeded job detail, click View Profile for organisation 700000000000000000000011.</x:v>
+      </x:c>
+      <x:c r="S14" s="41" t="str">
+        <x:v>The organisation profile loads with zero or more listings.</x:v>
+      </x:c>
+      <x:c r="T14" s="41" t="str">
+        <x:v>Cannot return null for non-nullable field Organisation.marketplaceListings.</x:v>
+      </x:c>
+      <x:c r="U14" s="41" t="str">
+        <x:v>apps/subgraph-classifieds/src/resolvers/index.spec.ts</x:v>
+      </x:c>
+      <x:c r="V14" s="41"/>
+      <x:c r="W14" s="41" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X14" s="41" t="str">
+        <x:v>The resolver index assigned only jobResolvers.Organisation and discarded the marketplace field resolver.</x:v>
+      </x:c>
+      <x:c r="Y14" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z14" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA14" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB14" s="41" t="str">
+        <x:v>EXEC-0059</x:v>
+      </x:c>
+      <x:c r="AC14" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD14" s="41" t="str">
+        <x:v>Merged job and marketplace Organisation resolver maps and added a regression test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="41" t="str">
+        <x:v>BUG-0010</x:v>
+      </x:c>
+      <x:c r="B15" s="41" t="str">
+        <x:v>Frontend exposed raw GraphQL and backend errors</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>ORG-005</x:v>
+      </x:c>
+      <x:c r="D15" s="41" t="str">
+        <x:v>EXEC-0059</x:v>
+      </x:c>
+      <x:c r="E15" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F15" s="41" t="str">
+        <x:v>Error Handling</x:v>
+      </x:c>
+      <x:c r="G15" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H15" s="41" t="str">
+        <x:v>Public and member page states</x:v>
+      </x:c>
+      <x:c r="I15" s="41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J15" s="41" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K15" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L15" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M15" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N15" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O15" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P15" s="66" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q15" s="41" t="str">
+        <x:v>Technical GraphQL completion messages and backend details were rendered directly to end users.</x:v>
+      </x:c>
+      <x:c r="R15" s="41" t="str">
+        <x:v>Force a GraphQL failure on a public/detail/member route and inspect the page error state.</x:v>
+      </x:c>
+      <x:c r="S15" s="41" t="str">
+        <x:v>Users receive safe actionable copy; technical details remain in development diagnostics.</x:v>
+      </x:c>
+      <x:c r="T15" s="41" t="str">
+        <x:v>Raw error.message text appeared below user-facing headings.</x:v>
+      </x:c>
+      <x:c r="U15" s="41" t="str">
+        <x:v>apps/christian-listing/src/lib/user-safe-error.ts; updated page states</x:v>
+      </x:c>
+      <x:c r="V15" s="41"/>
+      <x:c r="W15" s="41"/>
+      <x:c r="X15" s="41" t="str">
+        <x:v>Pages independently rendered Apollo and mutation exception messages without a presentation boundary.</x:v>
+      </x:c>
+      <x:c r="Y15" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z15" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA15" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB15" s="41"/>
+      <x:c r="AC15" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD15" s="41" t="str">
+        <x:v>Added shared safe-error mapping and replaced raw error rendering across the Christian Listings portal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" s="41" t="str">
+        <x:v>BUG-0011</x:v>
+      </x:c>
+      <x:c r="B16" s="41" t="str">
+        <x:v>Organisation contact links displayed __typename</x:v>
+      </x:c>
+      <x:c r="C16" s="41" t="str">
+        <x:v>ORG-005</x:v>
+      </x:c>
+      <x:c r="D16" s="41" t="str">
+        <x:v>EXEC-0059</x:v>
+      </x:c>
+      <x:c r="E16" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F16" s="41" t="str">
+        <x:v>Organisation Profile</x:v>
+      </x:c>
+      <x:c r="G16" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H16" s="41" t="str">
+        <x:v>Contact and social links</x:v>
+      </x:c>
+      <x:c r="I16" s="41" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J16" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K16" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L16" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M16" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N16" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O16" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P16" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q16" s="41" t="str">
+        <x:v>A contact capsule labelled __typename appeared beside the organisation phone number.</x:v>
+      </x:c>
+      <x:c r="R16" s="41" t="str">
+        <x:v>Open organisation 700000000000000000000011 and inspect Contact and social links.</x:v>
+      </x:c>
+      <x:c r="S16" s="41" t="str">
+        <x:v>Only supported social/contact fields render as capsules.</x:v>
+      </x:c>
+      <x:c r="T16" s="41" t="str">
+        <x:v>GraphQL metadata was iterated as if it were a social network.</x:v>
+      </x:c>
+      <x:c r="U16" s="41" t="str">
+        <x:v>apps/christian-listing/src/pages/OrganisationProfilePage.tsx</x:v>
+      </x:c>
+      <x:c r="V16" s="41"/>
+      <x:c r="W16" s="41" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X16" s="41" t="str">
+        <x:v>Object.entries included Apollo-added __typename metadata.</x:v>
+      </x:c>
+      <x:c r="Y16" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z16" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA16" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB16" s="41"/>
+      <x:c r="AC16" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD16" s="41" t="str">
+        <x:v>Replaced generic object iteration with an allowlist of supported social networks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="41" t="str">
+        <x:v>BUG-0012</x:v>
+      </x:c>
+      <x:c r="B17" s="41" t="str">
+        <x:v>Dashboard pages were obscured by the fixed navbar</x:v>
+      </x:c>
+      <x:c r="C17" s="41" t="str">
+        <x:v>JOB-006</x:v>
+      </x:c>
+      <x:c r="D17" s="41" t="str">
+        <x:v>EXEC-0031</x:v>
+      </x:c>
+      <x:c r="E17" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F17" s="41" t="str">
+        <x:v>Member Dashboard</x:v>
+      </x:c>
+      <x:c r="G17" s="41" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H17" s="41" t="str">
+        <x:v>Dashboard page shells</x:v>
+      </x:c>
+      <x:c r="I17" s="41" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J17" s="41" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K17" s="41" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L17" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M17" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N17" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O17" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P17" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q17" s="41" t="str">
+        <x:v>Dashboard and member subpage content began underneath the fixed navbar.</x:v>
+      </x:c>
+      <x:c r="R17" s="41" t="str">
+        <x:v>Open /dashboard and each member dashboard route at desktop width.</x:v>
+      </x:c>
+      <x:c r="S17" s="41" t="str">
+        <x:v>Headings and controls begin below the navbar on every dashboard route.</x:v>
+      </x:c>
+      <x:c r="T17" s="41" t="str">
+        <x:v>Top content was overlapped by navigation.</x:v>
+      </x:c>
+      <x:c r="U17" s="41" t="str">
+        <x:v>DashboardPage.tsx; MyApplicationsPage.tsx; SavedItemsPage.tsx; FollowingPage.tsx; MessagingPage.tsx</x:v>
+      </x:c>
+      <x:c r="V17" s="41"/>
+      <x:c r="W17" s="41"/>
+      <x:c r="X17" s="41" t="str">
+        <x:v>Dashboard route containers did not share the fixed-header spacing contract.</x:v>
+      </x:c>
+      <x:c r="Y17" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z17" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA17" s="41" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="AB17" s="41"/>
+      <x:c r="AC17" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD17" s="41" t="str">
+        <x:v>Applied consistent pt-28 page-shell spacing to the dashboard and member subpages.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" s="41" t="str">
+        <x:v>BUG-0013</x:v>
+      </x:c>
+      <x:c r="B18" s="41" t="str">
+        <x:v>Stale service worker caused repeated job-application deep-link requests</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>JOB-004</x:v>
+      </x:c>
+      <x:c r="D18" s="41" t="str">
+        <x:v>EXEC-0029</x:v>
+      </x:c>
+      <x:c r="E18" s="41" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F18" s="41" t="str">
+        <x:v>Job Applications</x:v>
+      </x:c>
+      <x:c r="G18" s="41" t="str">
+        <x:v>Deployment / Configuration</x:v>
+      </x:c>
+      <x:c r="H18" s="41" t="str">
+        <x:v>Development service worker and SPA fallback</x:v>
+      </x:c>
+      <x:c r="I18" s="41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J18" s="41" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K18" s="41" t="str">
+        <x:v>Closed</x:v>
+      </x:c>
+      <x:c r="L18" s="41" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M18" s="41" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N18" s="41" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O18" s="41" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P18" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q18" s="41" t="str">
+        <x:v>The application page repeatedly requested the organisation pathname; DevTools showed service-worker.js as initiator and 404 responses.</x:v>
+      </x:c>
+      <x:c r="R18" s="41" t="str">
+        <x:v>Open /jobs/700000000000000000000032/apply with a stale localhost service worker registered.</x:v>
+      </x:c>
+      <x:c r="S18" s="41" t="str">
+        <x:v>The SPA deep link renders once and no worker intercepts development navigation.</x:v>
+      </x:c>
+      <x:c r="T18" s="41" t="str">
+        <x:v>A legacy worker intercepted requests and the dev server returned 404 for history paths.</x:v>
+      </x:c>
+      <x:c r="U18" s="41" t="str">
+        <x:v>Browser Network initiator service-worker.js:56; main.tsx; webpack.config.js</x:v>
+      </x:c>
+      <x:c r="V18" s="41"/>
+      <x:c r="W18" s="41" t="str">
+        <x:v>Job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X18" s="41" t="str">
+        <x:v>A stale service-worker registration controlled localhost while the dev server lacked an explicit history fallback.</x:v>
+      </x:c>
+      <x:c r="Y18" s="41" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z18" s="41" t="str">
+        <x:v>Local working tree (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA18" s="41" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="AB18" s="41" t="str">
+        <x:v>EXEC-0029</x:v>
+      </x:c>
+      <x:c r="AC18" s="66" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD18" s="41" t="str">
+        <x:v>Development bootstrap unregisters stale workers once and Webpack serves history API fallbacks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="39"/>
@@ -28973,7 +29784,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246d7daf0c0b4ef8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf93190f72c84db9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32147,7 +32958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d25ca889f7b4171"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378247fe0c2a472f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32294,15 +33105,21 @@
       <x:c r="C6" s="39" t="str">
         <x:v>Local</x:v>
       </x:c>
-      <x:c r="D6" s="39" t="str"/>
-      <x:c r="E6" s="43" t="str"/>
-      <x:c r="F6" s="43" t="str"/>
-      <x:c r="G6" s="39" t="str"/>
+      <x:c r="D6" s="39" t="str">
+        <x:v>54ad9af + local fixes</x:v>
+      </x:c>
+      <x:c r="E6" s="43" t="str">
+        <x:v>18 Jul 2026</x:v>
+      </x:c>
+      <x:c r="F6" s="43"/>
+      <x:c r="G6" s="39" t="str">
+        <x:v>Product + Engineering</x:v>
+      </x:c>
       <x:c r="H6" s="39" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I6" s="39" t="str">
-        <x:v>All implemented P0/P1 flows</x:v>
+        <x:v>Initial E2E bug-fix cycle; full P0/P1 execution remains in progress</x:v>
       </x:c>
       <x:c r="J6" s="39" t="str">
         <x:v>Stack healthy and seed data loaded</x:v>
@@ -32316,10 +33133,10 @@
       </x:c>
       <x:c r="M6" s="39" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P1",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$A$6:$A$505,"&lt;&gt;")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="N6" s="39" t="str">
-        <x:v>Use one execution row per flow variant.</x:v>
+        <x:v>13 fixed defects recorded; 7 confirmed by follow-up retest and 6 ready for formal retest.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -35525,7 +36342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc45e74b679df41d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90c791caebef4591"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Job applications, organisation dashboard and creation workflows
</commit_message>
<xml_diff>
--- a/outputs/e2e-testing/E2E-TEST-TRACKER.xlsx
+++ b/outputs/e2e-testing/E2E-TEST-TRACKER.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5dafdc1e154f4712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Register" sheetId="2" r:id="Rbe24463c8e894590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="3" r:id="R9d4f9a462fa44b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R2c1af0f23fb94d4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Checks" sheetId="5" r:id="Rc1afa44e317c4950"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="6" r:id="Rd1376a9d96ab4d4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists &amp; Config" sheetId="7" r:id="R3cd5fbac2517492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R09edff13767f4e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Register" sheetId="2" r:id="Re6aaa8a2ac27431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="3" r:id="R0df7edf1aae2472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R6fd5af6ec583471c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB Checks" sheetId="5" r:id="Ra1309c56cb1343bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="6" r:id="Rea11063a558d4ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists &amp; Config" sheetId="7" r:id="R87ede405f6004cba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -828,7 +828,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4f89dd0203340d1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra6fb2bbb928f4986"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -858,7 +858,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R70729041dc8446e8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd91aaf4396fe417e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -929,8 +929,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:AD18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:AD18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DefectsTable" displayName="DefectsTable" ref="A5:AD27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:AD27"/>
   <x:tableColumns count="30">
     <x:tableColumn id="1" name="Defect ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1310,7 +1310,7 @@
       </x:c>
       <x:c r="E5" s="48" t="n">
         <x:f>COUNTIF('Defects'!$K$6:$K$505,"New")+COUNTIF('Defects'!$K$6:$K$505,"Triaged")+COUNTIF('Defects'!$K$6:$K$505,"In Progress")+COUNTIF('Defects'!$K$6:$K$505,"Ready for Retest")+COUNTIF('Defects'!$K$6:$K$505,"Reopened")+COUNTIF('Defects'!$K$6:$K$505,"Blocked")</x:f>
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F5" s="34"/>
       <x:c r="G5" s="34"/>
@@ -1335,7 +1335,7 @@
       </x:c>
       <x:c r="E6" s="48" t="n">
         <x:f>COUNTIFS('Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$I$6:$I$505,"P0",'Defects'!$K$6:$K$505,"&lt;&gt;Closed")+COUNTIFS('Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$I$6:$I$505,"P1",'Defects'!$K$6:$K$505,"&lt;&gt;Closed")</x:f>
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F6" s="34"/>
       <x:c r="G6" s="34"/>
@@ -1360,7 +1360,7 @@
       </x:c>
       <x:c r="E7" s="48" t="n">
         <x:f>COUNTIF('Defects'!$K$6:$K$505,"Ready for Retest")</x:f>
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F7" s="34"/>
       <x:c r="G7" s="34"/>
@@ -1527,7 +1527,7 @@
       </x:c>
       <x:c r="E15" s="53" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P0",'Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$K$6:$K$505,"&lt;&gt;Resolved")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F15" s="34"/>
       <x:c r="G15" s="34"/>
@@ -1552,7 +1552,7 @@
       </x:c>
       <x:c r="E16" s="53" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P1",'Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$K$6:$K$505,"&lt;&gt;Resolved")</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F16" s="34"/>
       <x:c r="G16" s="34"/>
@@ -1577,7 +1577,7 @@
       </x:c>
       <x:c r="E17" s="53" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P2",'Defects'!$A$6:$A$505,"&lt;&gt;",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$K$6:$K$505,"&lt;&gt;Resolved")</x:f>
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F17" s="34"/>
       <x:c r="G17" s="34"/>
@@ -1646,7 +1646,7 @@
     <x:cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="In Progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra172802743de41f8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9c34fe6ff364c31"/>
 </x:worksheet>
 </file>
 
@@ -7328,7 +7328,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad3e212d7cfd49a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5294a98d2ec04f90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8786,7 +8786,7 @@
       <x:c r="Q27" s="41" t="str"/>
       <x:c r="R27" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C27)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S27" s="39" t="str"/>
       <x:c r="T27" s="39" t="str"/>
@@ -9175,7 +9175,7 @@
       <x:c r="Q34" s="41" t="str"/>
       <x:c r="R34" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C34)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="S34" s="39" t="str">
         <x:v>BUG-0013</x:v>
@@ -9295,7 +9295,7 @@
       <x:c r="Q36" s="41" t="str"/>
       <x:c r="R36" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C36)</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="S36" s="39" t="str">
         <x:v>BUG-0012</x:v>
@@ -10126,7 +10126,7 @@
       <x:c r="Q51" s="41" t="str"/>
       <x:c r="R51" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C51)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S51" s="39" t="str"/>
       <x:c r="T51" s="39" t="str"/>
@@ -10686,7 +10686,7 @@
       <x:c r="Q61" s="41" t="str"/>
       <x:c r="R61" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C61)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S61" s="39" t="str"/>
       <x:c r="T61" s="39" t="str"/>
@@ -10741,7 +10741,7 @@
       <x:c r="Q62" s="41" t="str"/>
       <x:c r="R62" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C62)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S62" s="39" t="str"/>
       <x:c r="T62" s="39" t="str"/>
@@ -11246,7 +11246,7 @@
       <x:c r="Q71" s="41" t="str"/>
       <x:c r="R71" s="39" t="n">
         <x:f>COUNTIF('Defects'!$C$6:$C$505,C71)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S71" s="39" t="str"/>
       <x:c r="T71" s="39" t="str"/>
@@ -12759,7 +12759,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0412d6ce7e6d4b71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bdc17ead9b5475b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14169,292 +14169,794 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="39"/>
-      <x:c r="B19" s="39"/>
-      <x:c r="C19" s="39"/>
-      <x:c r="D19" s="39"/>
-      <x:c r="E19" s="39"/>
-      <x:c r="F19" s="39"/>
-      <x:c r="G19" s="39"/>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="39"/>
-      <x:c r="J19" s="39"/>
-      <x:c r="K19" s="39"/>
-      <x:c r="L19" s="39"/>
-      <x:c r="M19" s="39"/>
-      <x:c r="N19" s="39"/>
-      <x:c r="O19" s="39"/>
-      <x:c r="P19" s="43"/>
-      <x:c r="Q19" s="41"/>
-      <x:c r="R19" s="41"/>
-      <x:c r="S19" s="41"/>
-      <x:c r="T19" s="41"/>
-      <x:c r="U19" s="39"/>
+      <x:c r="A19" s="39" t="str">
+        <x:v>BUG-0014</x:v>
+      </x:c>
+      <x:c r="B19" s="39" t="str">
+        <x:v>Job detail retained Apply action after successful submission</x:v>
+      </x:c>
+      <x:c r="C19" s="39" t="str">
+        <x:v>JOB-004</x:v>
+      </x:c>
+      <x:c r="D19" s="39" t="str">
+        <x:v>EXEC-0029</x:v>
+      </x:c>
+      <x:c r="E19" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F19" s="39" t="str">
+        <x:v>Job Applications</x:v>
+      </x:c>
+      <x:c r="G19" s="39" t="str">
+        <x:v>UI / State</x:v>
+      </x:c>
+      <x:c r="H19" s="39" t="str">
+        <x:v>Job detail apply state</x:v>
+      </x:c>
+      <x:c r="I19" s="39" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J19" s="39" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K19" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L19" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M19" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N19" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O19" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P19" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q19" s="41" t="str">
+        <x:v>After submitting an application, the job detail page still offered Apply to Job.</x:v>
+      </x:c>
+      <x:c r="R19" s="41" t="str">
+        <x:v>Submit an application for job 700000000000000000000032, then return to its detail page.</x:v>
+      </x:c>
+      <x:c r="S19" s="41" t="str">
+        <x:v>The detail page shows Application Submitted and does not offer another application action.</x:v>
+      </x:c>
+      <x:c r="T19" s="41" t="str">
+        <x:v>Apply to Job remained visible after a successful submission.</x:v>
+      </x:c>
+      <x:c r="U19" s="39" t="str">
+        <x:v>JobDetailsPage.tsx; myJobApplication query</x:v>
+      </x:c>
       <x:c r="V19" s="39"/>
-      <x:c r="W19" s="39"/>
-      <x:c r="X19" s="39"/>
-      <x:c r="Y19" s="39"/>
-      <x:c r="Z19" s="39"/>
-      <x:c r="AA19" s="39"/>
+      <x:c r="W19" s="39" t="str">
+        <x:v>Job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X19" s="39" t="str">
+        <x:v>The detail query did not request the current member application state.</x:v>
+      </x:c>
+      <x:c r="Y19" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z19" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA19" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB19" s="39"/>
-      <x:c r="AC19" s="43"/>
-      <x:c r="AD19" s="39"/>
+      <x:c r="AC19" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD19" s="39" t="str">
+        <x:v>Queried myJobApplication and render a submitted state when an application exists.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="39"/>
-      <x:c r="B20" s="39"/>
-      <x:c r="C20" s="39"/>
-      <x:c r="D20" s="39"/>
-      <x:c r="E20" s="39"/>
-      <x:c r="F20" s="39"/>
-      <x:c r="G20" s="39"/>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="39"/>
-      <x:c r="J20" s="39"/>
-      <x:c r="K20" s="39"/>
-      <x:c r="L20" s="39"/>
-      <x:c r="M20" s="39"/>
-      <x:c r="N20" s="39"/>
-      <x:c r="O20" s="39"/>
-      <x:c r="P20" s="43"/>
-      <x:c r="Q20" s="41"/>
-      <x:c r="R20" s="41"/>
-      <x:c r="S20" s="41"/>
-      <x:c r="T20" s="41"/>
-      <x:c r="U20" s="39"/>
+      <x:c r="A20" s="39" t="str">
+        <x:v>BUG-0015</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="str">
+        <x:v>Member applications query returned empty for a valid application</x:v>
+      </x:c>
+      <x:c r="C20" s="39" t="str">
+        <x:v>JOB-006</x:v>
+      </x:c>
+      <x:c r="D20" s="39" t="str">
+        <x:v>EXEC-0031</x:v>
+      </x:c>
+      <x:c r="E20" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F20" s="39" t="str">
+        <x:v>Job Applications</x:v>
+      </x:c>
+      <x:c r="G20" s="39" t="str">
+        <x:v>API / GraphQL</x:v>
+      </x:c>
+      <x:c r="H20" s="39" t="str">
+        <x:v>User.jobApplications federation resolver</x:v>
+      </x:c>
+      <x:c r="I20" s="39" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J20" s="39" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K20" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L20" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M20" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N20" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O20" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P20" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q20" s="41" t="str">
+        <x:v>The authenticated member had a stored application, but me.jobApplications returned an empty array.</x:v>
+      </x:c>
+      <x:c r="R20" s="41" t="str">
+        <x:v>Submit a job application, then query me { id jobApplications { id } }.</x:v>
+      </x:c>
+      <x:c r="S20" s="41" t="str">
+        <x:v>The application associated with the Firebase principal is returned exactly once.</x:v>
+      </x:c>
+      <x:c r="T20" s="41" t="str">
+        <x:v>The query returned jobApplications: [] despite the persisted submission.</x:v>
+      </x:c>
+      <x:c r="U20" s="39" t="str">
+        <x:v>job-application.resolver.ts; user-federation.resolver.spec.ts</x:v>
+      </x:c>
       <x:c r="V20" s="39"/>
-      <x:c r="W20" s="39"/>
-      <x:c r="X20" s="39"/>
-      <x:c r="Y20" s="39"/>
-      <x:c r="Z20" s="39"/>
-      <x:c r="AA20" s="39"/>
+      <x:c r="W20" s="39" t="str">
+        <x:v>Member 6a5b4266de3d4b836e4a5a4d; job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X20" s="39" t="str">
+        <x:v>The federated User resolver compared JobApplication.userFirebaseUid with the Mongo User.id.</x:v>
+      </x:c>
+      <x:c r="Y20" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z20" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA20" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB20" s="39"/>
-      <x:c r="AC20" s="43"/>
-      <x:c r="AD20" s="39"/>
+      <x:c r="AC20" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD20" s="39" t="str">
+        <x:v>Resolved applications and listings by User.firebaseUid and added regression coverage.</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="39"/>
-      <x:c r="B21" s="39"/>
-      <x:c r="C21" s="39"/>
-      <x:c r="D21" s="39"/>
-      <x:c r="E21" s="39"/>
-      <x:c r="F21" s="39"/>
-      <x:c r="G21" s="39"/>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="39"/>
-      <x:c r="J21" s="39"/>
-      <x:c r="K21" s="39"/>
-      <x:c r="L21" s="39"/>
-      <x:c r="M21" s="39"/>
-      <x:c r="N21" s="39"/>
-      <x:c r="O21" s="39"/>
-      <x:c r="P21" s="43"/>
-      <x:c r="Q21" s="41"/>
-      <x:c r="R21" s="41"/>
-      <x:c r="S21" s="41"/>
-      <x:c r="T21" s="41"/>
-      <x:c r="U21" s="39"/>
+      <x:c r="A21" s="39" t="str">
+        <x:v>BUG-0016</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="str">
+        <x:v>Application history failed on null JobListing.title</x:v>
+      </x:c>
+      <x:c r="C21" s="39" t="str">
+        <x:v>JOB-006</x:v>
+      </x:c>
+      <x:c r="D21" s="39" t="str">
+        <x:v>EXEC-0031</x:v>
+      </x:c>
+      <x:c r="E21" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F21" s="39" t="str">
+        <x:v>Job Applications</x:v>
+      </x:c>
+      <x:c r="G21" s="39" t="str">
+        <x:v>API / GraphQL</x:v>
+      </x:c>
+      <x:c r="H21" s="39" t="str">
+        <x:v>JobApplication.listing</x:v>
+      </x:c>
+      <x:c r="I21" s="39" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="J21" s="39" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K21" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L21" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M21" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N21" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O21" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P21" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q21" s="41" t="str">
+        <x:v>After fixing application lookup, me became null because listing.title could not complete its non-null contract.</x:v>
+      </x:c>
+      <x:c r="R21" s="41" t="str">
+        <x:v>Query me.jobApplications.listing.title for a stored application.</x:v>
+      </x:c>
+      <x:c r="S21" s="41" t="str">
+        <x:v>Each application returns a hydrated local job listing with its required title.</x:v>
+      </x:c>
+      <x:c r="T21" s="41" t="str">
+        <x:v>GraphQL returned Cannot return null for non-nullable field JobListing.title.</x:v>
+      </x:c>
+      <x:c r="U21" s="39" t="str">
+        <x:v>GraphQL response; job-application.resolver.ts</x:v>
+      </x:c>
       <x:c r="V21" s="39"/>
-      <x:c r="W21" s="39"/>
-      <x:c r="X21" s="39"/>
-      <x:c r="Y21" s="39"/>
-      <x:c r="Z21" s="39"/>
-      <x:c r="AA21" s="39"/>
+      <x:c r="W21" s="39" t="str">
+        <x:v>Job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X21" s="39" t="str">
+        <x:v>JobApplication.listing returned only an entity reference that did not hydrate required local fields in this query path.</x:v>
+      </x:c>
+      <x:c r="Y21" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z21" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA21" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB21" s="39"/>
-      <x:c r="AC21" s="43"/>
-      <x:c r="AD21" s="39"/>
+      <x:c r="AC21" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD21" s="39" t="str">
+        <x:v>Hydrated the JobListing through the classifieds mapper before GraphQL completion.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="39"/>
-      <x:c r="B22" s="39"/>
-      <x:c r="C22" s="39"/>
-      <x:c r="D22" s="39"/>
-      <x:c r="E22" s="39"/>
-      <x:c r="F22" s="39"/>
-      <x:c r="G22" s="39"/>
-      <x:c r="H22" s="39"/>
-      <x:c r="I22" s="39"/>
-      <x:c r="J22" s="39"/>
-      <x:c r="K22" s="39"/>
-      <x:c r="L22" s="39"/>
-      <x:c r="M22" s="39"/>
-      <x:c r="N22" s="39"/>
-      <x:c r="O22" s="39"/>
-      <x:c r="P22" s="43"/>
-      <x:c r="Q22" s="41"/>
-      <x:c r="R22" s="41"/>
-      <x:c r="S22" s="41"/>
-      <x:c r="T22" s="41"/>
-      <x:c r="U22" s="39"/>
+      <x:c r="A22" s="39" t="str">
+        <x:v>BUG-0017</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="str">
+        <x:v>Submitted application response could not be reviewed</x:v>
+      </x:c>
+      <x:c r="C22" s="39" t="str">
+        <x:v>JOB-006</x:v>
+      </x:c>
+      <x:c r="D22" s="39" t="str">
+        <x:v>EXEC-0031</x:v>
+      </x:c>
+      <x:c r="E22" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F22" s="39" t="str">
+        <x:v>Member Dashboard</x:v>
+      </x:c>
+      <x:c r="G22" s="39" t="str">
+        <x:v>UI</x:v>
+      </x:c>
+      <x:c r="H22" s="39" t="str">
+        <x:v>My Applications</x:v>
+      </x:c>
+      <x:c r="I22" s="39" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J22" s="39" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K22" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L22" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M22" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N22" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O22" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P22" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q22" s="41" t="str">
+        <x:v>The applications dashboard showed status but offered no way to inspect the submitted answers.</x:v>
+      </x:c>
+      <x:c r="R22" s="41" t="str">
+        <x:v>Open /dashboard/applications after submitting an internal job application.</x:v>
+      </x:c>
+      <x:c r="S22" s="41" t="str">
+        <x:v>A member can open a read-only view of every submitted field.</x:v>
+      </x:c>
+      <x:c r="T22" s="41" t="str">
+        <x:v>Only the summary row and application status were available.</x:v>
+      </x:c>
+      <x:c r="U22" s="39" t="str">
+        <x:v>MyApplicationsPage.tsx</x:v>
+      </x:c>
       <x:c r="V22" s="39"/>
-      <x:c r="W22" s="39"/>
-      <x:c r="X22" s="39"/>
-      <x:c r="Y22" s="39"/>
-      <x:c r="Z22" s="39"/>
-      <x:c r="AA22" s="39"/>
+      <x:c r="W22" s="39" t="str">
+        <x:v>Job 700000000000000000000032</x:v>
+      </x:c>
+      <x:c r="X22" s="39" t="str">
+        <x:v>The dashboard query and UI were designed only for status summaries.</x:v>
+      </x:c>
+      <x:c r="Y22" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z22" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA22" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB22" s="39"/>
-      <x:c r="AC22" s="43"/>
-      <x:c r="AD22" s="39"/>
+      <x:c r="AC22" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD22" s="39" t="str">
+        <x:v>Added submitted fields to the query and an accessible read-only response modal.</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="39"/>
-      <x:c r="B23" s="39"/>
-      <x:c r="C23" s="39"/>
-      <x:c r="D23" s="39"/>
-      <x:c r="E23" s="39"/>
-      <x:c r="F23" s="39"/>
-      <x:c r="G23" s="39"/>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="39"/>
-      <x:c r="J23" s="39"/>
-      <x:c r="K23" s="39"/>
-      <x:c r="L23" s="39"/>
-      <x:c r="M23" s="39"/>
-      <x:c r="N23" s="39"/>
-      <x:c r="O23" s="39"/>
-      <x:c r="P23" s="43"/>
-      <x:c r="Q23" s="41"/>
-      <x:c r="R23" s="41"/>
-      <x:c r="S23" s="41"/>
-      <x:c r="T23" s="41"/>
-      <x:c r="U23" s="39"/>
+      <x:c r="A23" s="39" t="str">
+        <x:v>BUG-0018</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="str">
+        <x:v>Organisation social connection add action was inert</x:v>
+      </x:c>
+      <x:c r="C23" s="39" t="str">
+        <x:v>ORG-003</x:v>
+      </x:c>
+      <x:c r="D23" s="39" t="str">
+        <x:v>EXEC-0057</x:v>
+      </x:c>
+      <x:c r="E23" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F23" s="39" t="str">
+        <x:v>Organisation Dashboard</x:v>
+      </x:c>
+      <x:c r="G23" s="39" t="str">
+        <x:v>UI / Navigation</x:v>
+      </x:c>
+      <x:c r="H23" s="39" t="str">
+        <x:v>Social Connection</x:v>
+      </x:c>
+      <x:c r="I23" s="39" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J23" s="39" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K23" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L23" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M23" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N23" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O23" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P23" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q23" s="41" t="str">
+        <x:v>The plus control in Social Connection had no click behaviour.</x:v>
+      </x:c>
+      <x:c r="R23" s="41" t="str">
+        <x:v>Sign in as an organisation owner, open /org, and click the plus control.</x:v>
+      </x:c>
+      <x:c r="S23" s="41" t="str">
+        <x:v>The user is taken directly to editable organisation social-link settings.</x:v>
+      </x:c>
+      <x:c r="T23" s="41" t="str">
+        <x:v>The control did nothing.</x:v>
+      </x:c>
+      <x:c r="U23" s="39" t="str">
+        <x:v>OrgOverviewPage.tsx; OrgSettingsPage.tsx</x:v>
+      </x:c>
       <x:c r="V23" s="39"/>
-      <x:c r="W23" s="39"/>
-      <x:c r="X23" s="39"/>
-      <x:c r="Y23" s="39"/>
-      <x:c r="Z23" s="39"/>
-      <x:c r="AA23" s="39"/>
+      <x:c r="W23" s="39" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X23" s="39" t="str">
+        <x:v>The control was a visual button without navigation or a form target.</x:v>
+      </x:c>
+      <x:c r="Y23" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z23" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA23" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB23" s="39"/>
-      <x:c r="AC23" s="43"/>
-      <x:c r="AD23" s="39"/>
+      <x:c r="AC23" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD23" s="39" t="str">
+        <x:v>Linked it to /org/settings#social-links, added anchored scrolling, and made existing social capsules actionable.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="39"/>
-      <x:c r="B24" s="39"/>
-      <x:c r="C24" s="39"/>
-      <x:c r="D24" s="39"/>
-      <x:c r="E24" s="39"/>
-      <x:c r="F24" s="39"/>
-      <x:c r="G24" s="39"/>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="39"/>
-      <x:c r="J24" s="39"/>
-      <x:c r="K24" s="39"/>
-      <x:c r="L24" s="39"/>
-      <x:c r="M24" s="39"/>
-      <x:c r="N24" s="39"/>
-      <x:c r="O24" s="39"/>
-      <x:c r="P24" s="43"/>
-      <x:c r="Q24" s="41"/>
-      <x:c r="R24" s="41"/>
-      <x:c r="S24" s="41"/>
-      <x:c r="T24" s="41"/>
-      <x:c r="U24" s="39"/>
+      <x:c r="A24" s="39" t="str">
+        <x:v>BUG-0019</x:v>
+      </x:c>
+      <x:c r="B24" s="39" t="str">
+        <x:v>Organisation overview omitted marketplace messages</x:v>
+      </x:c>
+      <x:c r="C24" s="39" t="str">
+        <x:v>MSG-002</x:v>
+      </x:c>
+      <x:c r="D24" s="39" t="str">
+        <x:v>EXEC-0046</x:v>
+      </x:c>
+      <x:c r="E24" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F24" s="39" t="str">
+        <x:v>Organisation Dashboard</x:v>
+      </x:c>
+      <x:c r="G24" s="39" t="str">
+        <x:v>UI / GraphQL</x:v>
+      </x:c>
+      <x:c r="H24" s="39" t="str">
+        <x:v>Marketplace Messages</x:v>
+      </x:c>
+      <x:c r="I24" s="39" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J24" s="39" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K24" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L24" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M24" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N24" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O24" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P24" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q24" s="41" t="str">
+        <x:v>The organisation overview had no marketplace buyer-message component despite the seller inbox being implemented.</x:v>
+      </x:c>
+      <x:c r="R24" s="41" t="str">
+        <x:v>Open /org and inspect the dashboard beneath the listings table.</x:v>
+      </x:c>
+      <x:c r="S24" s="41" t="str">
+        <x:v>Recent buyer conversations, unread counts, and inbox navigation are visible.</x:v>
+      </x:c>
+      <x:c r="T24" s="41" t="str">
+        <x:v>The dashboard grid reserved an empty column and exposed no conversation summary.</x:v>
+      </x:c>
+      <x:c r="U24" s="39" t="str">
+        <x:v>OrgOverviewPage.tsx; myMessageThreads(role: SELLER)</x:v>
+      </x:c>
       <x:c r="V24" s="39"/>
-      <x:c r="W24" s="39"/>
-      <x:c r="X24" s="39"/>
-      <x:c r="Y24" s="39"/>
-      <x:c r="Z24" s="39"/>
-      <x:c r="AA24" s="39"/>
+      <x:c r="W24" s="39" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X24" s="39" t="str">
+        <x:v>The seller messaging route existed but was never composed into the overview.</x:v>
+      </x:c>
+      <x:c r="Y24" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z24" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA24" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB24" s="39"/>
-      <x:c r="AC24" s="43"/>
-      <x:c r="AD24" s="39"/>
+      <x:c r="AC24" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD24" s="39" t="str">
+        <x:v>Added a live recent-conversation panel with loading, empty, error, unread, detail, and inbox states.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="39"/>
-      <x:c r="B25" s="39"/>
-      <x:c r="C25" s="39"/>
-      <x:c r="D25" s="39"/>
-      <x:c r="E25" s="39"/>
-      <x:c r="F25" s="39"/>
-      <x:c r="G25" s="39"/>
-      <x:c r="H25" s="39"/>
-      <x:c r="I25" s="39"/>
-      <x:c r="J25" s="39"/>
-      <x:c r="K25" s="39"/>
-      <x:c r="L25" s="39"/>
-      <x:c r="M25" s="39"/>
-      <x:c r="N25" s="39"/>
-      <x:c r="O25" s="39"/>
-      <x:c r="P25" s="43"/>
-      <x:c r="Q25" s="41"/>
-      <x:c r="R25" s="41"/>
-      <x:c r="S25" s="41"/>
-      <x:c r="T25" s="41"/>
-      <x:c r="U25" s="39"/>
+      <x:c r="A25" s="39" t="str">
+        <x:v>BUG-0020</x:v>
+      </x:c>
+      <x:c r="B25" s="39" t="str">
+        <x:v>View All Notifications action was inert</x:v>
+      </x:c>
+      <x:c r="C25" s="39" t="str">
+        <x:v>NOT-001</x:v>
+      </x:c>
+      <x:c r="D25" s="39" t="str">
+        <x:v>EXEC-0066</x:v>
+      </x:c>
+      <x:c r="E25" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F25" s="39" t="str">
+        <x:v>Organisation Dashboard</x:v>
+      </x:c>
+      <x:c r="G25" s="39" t="str">
+        <x:v>UI / Navigation</x:v>
+      </x:c>
+      <x:c r="H25" s="39" t="str">
+        <x:v>Notification Centre</x:v>
+      </x:c>
+      <x:c r="I25" s="39" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J25" s="39" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K25" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L25" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M25" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N25" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O25" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P25" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q25" s="41" t="str">
+        <x:v>The organisation overview notification footer did not open the notification centre.</x:v>
+      </x:c>
+      <x:c r="R25" s="41" t="str">
+        <x:v>Open /org and click View All Notifications.</x:v>
+      </x:c>
+      <x:c r="S25" s="41" t="str">
+        <x:v>The organisation notification centre opens at /org/notifications.</x:v>
+      </x:c>
+      <x:c r="T25" s="41" t="str">
+        <x:v>The button had no effect.</x:v>
+      </x:c>
+      <x:c r="U25" s="39" t="str">
+        <x:v>OrgOverviewPage.tsx; /org/notifications</x:v>
+      </x:c>
       <x:c r="V25" s="39"/>
-      <x:c r="W25" s="39"/>
-      <x:c r="X25" s="39"/>
-      <x:c r="Y25" s="39"/>
-      <x:c r="Z25" s="39"/>
-      <x:c r="AA25" s="39"/>
+      <x:c r="W25" s="39" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X25" s="39" t="str">
+        <x:v>The footer was rendered as a button without a click handler.</x:v>
+      </x:c>
+      <x:c r="Y25" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z25" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA25" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB25" s="39"/>
-      <x:c r="AC25" s="43"/>
-      <x:c r="AD25" s="39"/>
+      <x:c r="AC25" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD25" s="39" t="str">
+        <x:v>Replaced the inert control with a route link to the persistent notification centre.</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="39"/>
-      <x:c r="B26" s="39"/>
-      <x:c r="C26" s="39"/>
-      <x:c r="D26" s="39"/>
-      <x:c r="E26" s="39"/>
-      <x:c r="F26" s="39"/>
-      <x:c r="G26" s="39"/>
-      <x:c r="H26" s="39"/>
-      <x:c r="I26" s="39"/>
-      <x:c r="J26" s="39"/>
-      <x:c r="K26" s="39"/>
-      <x:c r="L26" s="39"/>
-      <x:c r="M26" s="39"/>
-      <x:c r="N26" s="39"/>
-      <x:c r="O26" s="39"/>
-      <x:c r="P26" s="43"/>
-      <x:c r="Q26" s="41"/>
-      <x:c r="R26" s="41"/>
-      <x:c r="S26" s="41"/>
-      <x:c r="T26" s="41"/>
-      <x:c r="U26" s="39"/>
+      <x:c r="A26" s="39" t="str">
+        <x:v>BUG-0021</x:v>
+      </x:c>
+      <x:c r="B26" s="39" t="str">
+        <x:v>Recurring event form submitted a zero-occurrence rule</x:v>
+      </x:c>
+      <x:c r="C26" s="39" t="str">
+        <x:v>EVT-009</x:v>
+      </x:c>
+      <x:c r="D26" s="39" t="str">
+        <x:v>EXEC-0022</x:v>
+      </x:c>
+      <x:c r="E26" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F26" s="39" t="str">
+        <x:v>Organisation Events</x:v>
+      </x:c>
+      <x:c r="G26" s="39" t="str">
+        <x:v>Validation / Backend Logic</x:v>
+      </x:c>
+      <x:c r="H26" s="39" t="str">
+        <x:v>Recurring event creation</x:v>
+      </x:c>
+      <x:c r="I26" s="39" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="J26" s="39" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K26" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L26" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M26" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N26" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O26" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P26" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q26" s="41" t="str">
+        <x:v>A weekly rule could end before its first selected weekday and reach createEvent with no possible occurrences.</x:v>
+      </x:c>
+      <x:c r="R26" s="41" t="str">
+        <x:v>Choose a start date, select a later weekday, set the series end before that weekday, and publish.</x:v>
+      </x:c>
+      <x:c r="S26" s="41" t="str">
+        <x:v>The form defaults to the event weekday and clearly blocks any end date before the first valid occurrence.</x:v>
+      </x:c>
+      <x:c r="T26" s="41" t="str">
+        <x:v>createEvent returned The recurrence rule does not produce any occurrences.</x:v>
+      </x:c>
+      <x:c r="U26" s="39" t="str">
+        <x:v>recurrence-form.ts; recurrence-form.spec.ts; OrgOverviewPage.tsx</x:v>
+      </x:c>
       <x:c r="V26" s="39"/>
       <x:c r="W26" s="39"/>
-      <x:c r="X26" s="39"/>
-      <x:c r="Y26" s="39"/>
-      <x:c r="Z26" s="39"/>
-      <x:c r="AA26" s="39"/>
+      <x:c r="X26" s="39" t="str">
+        <x:v>The form validated only that an end date existed, not that the selected schedule could occur before it.</x:v>
+      </x:c>
+      <x:c r="Y26" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z26" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA26" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB26" s="39"/>
-      <x:c r="AC26" s="43"/>
-      <x:c r="AD26" s="39"/>
+      <x:c r="AC26" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD26" s="39" t="str">
+        <x:v>Calculated the first valid weekly occurrence, set a schedule-aware minimum, displayed an inline warning, and disabled invalid submission.</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="39"/>
-      <x:c r="B27" s="39"/>
-      <x:c r="C27" s="39"/>
-      <x:c r="D27" s="39"/>
-      <x:c r="E27" s="39"/>
-      <x:c r="F27" s="39"/>
-      <x:c r="G27" s="39"/>
-      <x:c r="H27" s="39"/>
-      <x:c r="I27" s="39"/>
-      <x:c r="J27" s="39"/>
-      <x:c r="K27" s="39"/>
-      <x:c r="L27" s="39"/>
-      <x:c r="M27" s="39"/>
-      <x:c r="N27" s="39"/>
-      <x:c r="O27" s="39"/>
-      <x:c r="P27" s="43"/>
-      <x:c r="Q27" s="41"/>
-      <x:c r="R27" s="41"/>
-      <x:c r="S27" s="41"/>
-      <x:c r="T27" s="41"/>
-      <x:c r="U27" s="39"/>
+      <x:c r="A27" s="39" t="str">
+        <x:v>BUG-0022</x:v>
+      </x:c>
+      <x:c r="B27" s="39" t="str">
+        <x:v>Organisation manager pages lacked local create forms</x:v>
+      </x:c>
+      <x:c r="C27" s="39" t="str">
+        <x:v>ORG-002</x:v>
+      </x:c>
+      <x:c r="D27" s="39" t="str">
+        <x:v>EXEC-0056</x:v>
+      </x:c>
+      <x:c r="E27" s="39" t="str">
+        <x:v>Christian Listings</x:v>
+      </x:c>
+      <x:c r="F27" s="39" t="str">
+        <x:v>Organisation Dashboard</x:v>
+      </x:c>
+      <x:c r="G27" s="39" t="str">
+        <x:v>UI / Workflow</x:v>
+      </x:c>
+      <x:c r="H27" s="39" t="str">
+        <x:v>Events, listings, and jobs managers</x:v>
+      </x:c>
+      <x:c r="I27" s="39" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="J27" s="39" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K27" s="39" t="str">
+        <x:v>Ready for Retest</x:v>
+      </x:c>
+      <x:c r="L27" s="39" t="str">
+        <x:v>Local</x:v>
+      </x:c>
+      <x:c r="M27" s="39" t="str">
+        <x:v>Chrome</x:v>
+      </x:c>
+      <x:c r="N27" s="39" t="str">
+        <x:v>Product E2E</x:v>
+      </x:c>
+      <x:c r="O27" s="39" t="str">
+        <x:v>Engineering</x:v>
+      </x:c>
+      <x:c r="P27" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="Q27" s="41" t="str">
+        <x:v>Events, Listings, and Jobs manager pages required returning to Overview to create owned content.</x:v>
+      </x:c>
+      <x:c r="R27" s="41" t="str">
+        <x:v>Open /org/events, /org/listings, and /org/jobs and inspect below each table.</x:v>
+      </x:c>
+      <x:c r="S27" s="41" t="str">
+        <x:v>Each manager page contains its matching wired creation form and refreshes its table after success.</x:v>
+      </x:c>
+      <x:c r="T27" s="41" t="str">
+        <x:v>Creation was centralized on Overview and the manager pages ended after their tables.</x:v>
+      </x:c>
+      <x:c r="U27" s="39" t="str">
+        <x:v>OrgEventsPage.tsx; OrgListingsPage.tsx; OrgJobsPage.tsx</x:v>
+      </x:c>
       <x:c r="V27" s="39"/>
-      <x:c r="W27" s="39"/>
-      <x:c r="X27" s="39"/>
-      <x:c r="Y27" s="39"/>
-      <x:c r="Z27" s="39"/>
-      <x:c r="AA27" s="39"/>
+      <x:c r="W27" s="39" t="str">
+        <x:v>Organisation 700000000000000000000011</x:v>
+      </x:c>
+      <x:c r="X27" s="39" t="str">
+        <x:v>The creation forms were private to OrgOverviewPage and not composed into domain manager workflows.</x:v>
+      </x:c>
+      <x:c r="Y27" s="39" t="str">
+        <x:v>Pending commit (local fix)</x:v>
+      </x:c>
+      <x:c r="Z27" s="39" t="str">
+        <x:v>Local verified (19 Jul 2026)</x:v>
+      </x:c>
+      <x:c r="AA27" s="39" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
       <x:c r="AB27" s="39"/>
-      <x:c r="AC27" s="43"/>
-      <x:c r="AD27" s="39"/>
+      <x:c r="AC27" s="43" t="str">
+        <x:v>19 Jul 2026</x:v>
+      </x:c>
+      <x:c r="AD27" s="39" t="str">
+        <x:v>Exported and reused the existing forms below their respective tables with post-create refetch callbacks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="39"/>
@@ -29784,7 +30286,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf93190f72c84db9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9d5eb76fc784ed4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32958,7 +33460,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378247fe0c2a472f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81c3202910b84e70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33129,11 +33631,11 @@
       </x:c>
       <x:c r="L6" s="39" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P0",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$A$6:$A$505,"&lt;&gt;")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M6" s="39" t="n">
         <x:f>COUNTIFS('Defects'!$I$6:$I$505,"P1",'Defects'!$K$6:$K$505,"&lt;&gt;Closed",'Defects'!$A$6:$A$505,"&lt;&gt;")</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N6" s="39" t="str">
         <x:v>13 fixed defects recorded; 7 confirmed by follow-up retest and 6 ready for formal retest.</x:v>
@@ -36342,7 +36844,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90c791caebef4591"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb49043f1633e4ec9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>